<commit_message>
Changed powerpoint text colour to black
</commit_message>
<xml_diff>
--- a/Quantitative-Analysis.xlsx
+++ b/Quantitative-Analysis.xlsx
@@ -132,7 +132,7 @@
     <numFmt numFmtId="164" formatCode="General"/>
     <numFmt numFmtId="165" formatCode="#,##0.00"/>
   </numFmts>
-  <fonts count="6">
+  <fonts count="5">
     <font>
       <sz val="10"/>
       <color rgb="FF000000"/>
@@ -156,15 +156,8 @@
       <family val="0"/>
     </font>
     <font>
-      <sz val="10"/>
-      <color rgb="FFFFFFFF"/>
-      <name val="Arial"/>
-      <family val="0"/>
-      <charset val="1"/>
-    </font>
-    <font>
       <sz val="11"/>
-      <color rgb="FFFFFFFF"/>
+      <color rgb="FF000000"/>
       <name val="Arial"/>
       <family val="0"/>
       <charset val="1"/>
@@ -218,28 +211,24 @@
     <xf numFmtId="42" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
     <xf numFmtId="9" fontId="1" fillId="0" borderId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false"/>
   </cellStyleXfs>
-  <cellXfs count="6">
+  <cellXfs count="5">
     <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="false" applyBorder="false" applyAlignment="false" applyProtection="false">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="164" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="5" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="165" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
+    <xf numFmtId="165" fontId="0" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
-    <xf numFmtId="164" fontId="4" fillId="0" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="false" applyProtection="false">
-      <alignment horizontal="general" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
-      <protection locked="true" hidden="false"/>
-    </xf>
-    <xf numFmtId="165" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="false">
+    <xf numFmtId="165" fontId="0" fillId="2" borderId="0" xfId="0" applyFont="true" applyBorder="false" applyAlignment="true" applyProtection="true">
       <alignment horizontal="right" vertical="bottom" textRotation="0" wrapText="false" indent="0" shrinkToFit="false"/>
       <protection locked="true" hidden="false"/>
     </xf>
@@ -2799,7 +2788,7 @@
       <c r="B51" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="C51" s="4" t="n">
+      <c r="C51" s="1" t="n">
         <v>9</v>
       </c>
     </row>
@@ -2823,7 +2812,7 @@
       <c r="B54" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="C54" s="5" t="s">
+      <c r="C54" s="4" t="s">
         <v>31</v>
       </c>
     </row>
@@ -2952,7 +2941,7 @@
       <c r="B69" s="3" t="s">
         <v>27</v>
       </c>
-      <c r="C69" s="4" t="n">
+      <c r="C69" s="1" t="n">
         <v>8</v>
       </c>
     </row>
@@ -2976,7 +2965,7 @@
       <c r="B72" s="3" t="s">
         <v>30</v>
       </c>
-      <c r="C72" s="5" t="s">
+      <c r="C72" s="4" t="s">
         <v>33</v>
       </c>
     </row>

</xml_diff>